<commit_message>
docs: update m aterials spreadsheet
</commit_message>
<xml_diff>
--- a/hardware/materials.xlsx
+++ b/hardware/materials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshf\Documents\Code\USB_IR_Blaster\PCB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshf\Documents\Code\USB_IR_Blaster\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9814267-C47A-47AD-83EE-FF15C4386B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA45C1FE-7F93-46A2-A0A3-51A74267C9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FC31D8FB-3664-43EE-8E32-81502E5E38D7}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>Description</t>
   </si>
@@ -128,57 +128,6 @@
     <t>N-Channel 30 V 5.7A (Ta) 1.4W (Ta) Surface Mount SOT-23-3</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMCF1206FT6R20/2417449</t>
-  </si>
-  <si>
-    <t>RMCF1206FT6R20CT-ND</t>
-  </si>
-  <si>
-    <t>6.2 Ohms ±1% 0.25W, 1/4W Chip Resistor 1206 (3216 Metric) Automotive AEC-Q200 Thick Film</t>
-  </si>
-  <si>
-    <t>https://www.seielect.com/catalog/SEI-RMCF_RMCP.pdf</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/models/2417449?tab=ultralibrarian</t>
-  </si>
-  <si>
-    <t>RMCF1206FT6R20</t>
-  </si>
-  <si>
-    <t>Stackpole Electronics Inc</t>
-  </si>
-  <si>
-    <t>RMCF0805FT10K0CT-ND</t>
-  </si>
-  <si>
-    <t>RMCF0805FT10K0</t>
-  </si>
-  <si>
-    <t>10 kOhms ±1% 0.125W, 1/8W Chip Resistor 0805 (2012 Metric) Automotive AEC-Q200 Thick Film</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/models/1760676?tab=ultralibrarian</t>
-  </si>
-  <si>
-    <t>27.4 Ohms ±1% 0.25W, 1/4W Chip Resistor 1206 (3216 Metric) Automotive AEC-Q200 Thick Film</t>
-  </si>
-  <si>
-    <t>RMCF1206FT27R4CT-ND</t>
-  </si>
-  <si>
-    <t>RMCF1206FT27R4</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMCF1206FT27R4/1759794</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/models/1759794?tab=ultralibrarian</t>
-  </si>
-  <si>
     <t>2648-SC0914(13)CT-ND</t>
   </si>
   <si>
@@ -200,27 +149,9 @@
     <t>https://datasheets.raspberrypi.com/rp2040/rp2040-datasheet.pdf</t>
   </si>
   <si>
-    <t>https://www.mouser.com/ProductDetail/Texas-Instruments/TPSM828214SILR?qs=iLbezkQI%252BsibRGaNc1MtTA%3D%3D&amp;srsltid=AfmBOor4b8JqR77eR3sJy0Jea9YU8rNC9ZfQWXhB2TDbICdzHKXJhKOR</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/models/14124001?tab=ultralibrarian</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10A226MP8NUNE/3886932</t>
-  </si>
-  <si>
-    <t>22 µF ±20% 10V Ceramic Capacitor X5R 0603 (1608 Metric)</t>
-  </si>
-  <si>
-    <t>Switching Voltage Regulators 5.5-V input 1-A ste p-down module with i</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/cal-chip-electronics-inc/GMC10X7R475K10NT/24343641</t>
-  </si>
-  <si>
-    <t>4.7 µF ±10% 10V Ceramic Capacitor X7R 0603 (1608 Metric)</t>
-  </si>
-  <si>
     <t>FLASH - NOR Memory IC 128Mbit SPI - Quad I/O, QPI 133 MHz 8-SOIC</t>
   </si>
   <si>
@@ -230,25 +161,76 @@
     <t>https://www.digikey.com/en/products/detail/winbond-electronics/W25Q128JVSIQ/5803943</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/c-k/PTS636SM43SMTR-LFS/10071723</t>
-  </si>
-  <si>
-    <t>PTS636SM43SMTR LFS</t>
-  </si>
-  <si>
     <t>Tactile Switch SPST-NO Top Actuated Surface Mount</t>
   </si>
   <si>
-    <t>Button_Switch_SMD:SW_Push_6x3.5mm</t>
-  </si>
-  <si>
-    <t>https://www.mouser.com/ProductDetail/ABRACON/ABM8-272-T3?qs=QpmGXVUTftEj6miOiJBMxQ%3D%3D&amp;srsltid=AfmBOoreONVOH-K9twHGfSJF-Jpo5aXiXpnElmP-T8XmVjeTsv9DHJFU</t>
-  </si>
-  <si>
-    <t>Crystals Ultra Miniature Ceramic SMD Crystal</t>
-  </si>
-  <si>
     <t>ABM8-272-T3</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/TPSM828214SILR/14124001</t>
+  </si>
+  <si>
+    <t>296-TPSM828214SILRCT-ND</t>
+  </si>
+  <si>
+    <t>TPSM828214SILR</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/tpsm82821.pdf?HQS=dis-dk-null-digikeymode-dsf-pf-null-wwe&amp;ts=1783895550077&amp;ref_url=https%253A%252F%252Fwww.hkdcy.com</t>
+  </si>
+  <si>
+    <t>Winbond Electronics</t>
+  </si>
+  <si>
+    <t>W25Q128JVSIQ-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/models/5803943</t>
+  </si>
+  <si>
+    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/7161/256_W25Q128JV.pdf</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/abracon-llc/ABM8-272-T3/22472366</t>
+  </si>
+  <si>
+    <t>https://abracon.com/datasheets/ABM8-272-T3.pdf</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/models/22472366?tab=ultralibrarian</t>
+  </si>
+  <si>
+    <t>Abracon LLC</t>
+  </si>
+  <si>
+    <t>535-ABM8-272-T3CT-ND</t>
+  </si>
+  <si>
+    <t>https://omronfs.omron.com/en_US/ecb/products/pdf/en-b3u.pdf</t>
+  </si>
+  <si>
+    <t>12 MHz ±30ppm Crystal 10pF 50 Ohms 4-SMD, No Lead</t>
+  </si>
+  <si>
+    <t>Non-Isolated PoL Module DC DC Converter 1 Output 3.3V 1A 2.4V - 5.5V Input</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/omron-electronics-inc-emc-div/B3U-1000P/1534338</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/models/1534338</t>
+  </si>
+  <si>
+    <t>Aratas America LLC</t>
+  </si>
+  <si>
+    <t>B3U-1000P</t>
+  </si>
+  <si>
+    <t>SW1020CT-ND</t>
   </si>
 </sst>
 </file>
@@ -299,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -309,6 +291,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -644,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CDCC247-279C-4A9F-A582-D4D49D3E2219}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="15.265625" customWidth="1"/>
@@ -682,28 +667,28 @@
     </row>
     <row r="2" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="F2" s="2">
         <v>1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="142.5" x14ac:dyDescent="0.45">
@@ -749,7 +734,7 @@
         <v>17</v>
       </c>
       <c r="F4" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
@@ -784,44 +769,44 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="114" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" ht="185.25" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>30</v>
+        <v>58</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F6" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="114" x14ac:dyDescent="0.45">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>36</v>
+      <c r="D7" t="s">
+        <v>48</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>39</v>
@@ -830,100 +815,66 @@
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="A8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="114" x14ac:dyDescent="0.45">
+      <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="114" x14ac:dyDescent="0.45">
-      <c r="A8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8" s="2">
-        <v>2</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="213.75" x14ac:dyDescent="0.45">
-      <c r="A9" s="2" t="s">
-        <v>57</v>
+      <c r="B9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" t="s">
+        <v>63</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="114" x14ac:dyDescent="0.45">
-      <c r="A10" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="114" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="A12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" t="s">
-        <v>61</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="213.75" x14ac:dyDescent="0.45">
-      <c r="A14" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" t="s">
-        <v>69</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>67</v>
-      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="G10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>